<commit_message>
IANSEO scraper bugfixes and compiler scripts
</commit_message>
<xml_diff>
--- a/IANSEO scraper v2/urls.xlsx
+++ b/IANSEO scraper v2/urls.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C93DC1-7659-4640-9E13-701E419A3632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-4575" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-27660" yWindow="-3315" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Compiler bug fix and more urls
</commit_message>
<xml_diff>
--- a/IANSEO scraper v2/urls.xlsx
+++ b/IANSEO scraper v2/urls.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robog\Documents\GitHub\Archers-Against-Bigotry-Datahub-1\IANSEO scraper v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C93DC1-7659-4640-9E13-701E419A3632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2307564-C40E-4890-895E-D0FB645E50F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27660" yWindow="-3315" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="11380" windowHeight="13370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="117">
   <si>
     <t>https://www.ianseo.net/Details.php?toId=15718</t>
   </si>
@@ -311,6 +311,66 @@
   </si>
   <si>
     <t>https://www.ianseo.net/Details.php?toId=26274</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=26685</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=24037</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=24322</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=25594</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=25621</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=25557</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=25456</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=25279</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=23223</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=23222</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=21665</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=21887</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=21946</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=20178</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=21631</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=20716</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=21358</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=21454</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=20889</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=20803</t>
   </si>
 </sst>
 </file>
@@ -650,7 +710,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A97"/>
+  <dimension ref="A1:A117"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
@@ -1138,6 +1198,106 @@
         <v>96</v>
       </c>
     </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A106" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A108" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A109" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A110" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A111" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A112" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A113" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A114" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A115" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A116" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A117" t="s">
+        <v>116</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Finished the extra ianseo scraper and the compilers
</commit_message>
<xml_diff>
--- a/IANSEO scraper v2/urls.xlsx
+++ b/IANSEO scraper v2/urls.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robog\Documents\GitHub\Archers-Against-Bigotry-Datahub-1\IANSEO scraper v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2307564-C40E-4890-895E-D0FB645E50F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2071193B-FFE1-4A1C-83A8-FB340162CD1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="11380" windowHeight="13370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="740" yWindow="730" windowWidth="16800" windowHeight="9680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="187">
   <si>
     <t>https://www.ianseo.net/Details.php?toId=15718</t>
   </si>
@@ -371,16 +371,234 @@
   </si>
   <si>
     <t>https://www.ianseo.net/Details.php?toId=20803</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=20618</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=20130</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=20367</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=19866</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=18338</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=20029</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=17174</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=15801</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=16871</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=16878</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=16605</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=16682</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=16680</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=16741</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=15856</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=16532</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=16537</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=15998</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=16034</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=14805</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=15967</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=13521</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=12940</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=13398</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=12938</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=12939</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=12937</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=12289</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=12026</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=13003</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=12003</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=10377</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=10236</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=10374</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=10026</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=10027</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=10028</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=10040</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=9686</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=7058</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=6816</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=6963</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=6812</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=6813</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=6738</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=6948</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=6814</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=6470</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=6457</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=6381</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=6052</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=5355</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=5267</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=4914</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=5151</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=4915</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=5150</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=5066</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=4841</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=4770</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=3599</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=3731</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=3631</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=3656</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=3340</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=2546</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=2406</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=2085</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=929</t>
+  </si>
+  <si>
+    <t>https://www.ianseo.net/Details.php?toId=450</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -403,13 +621,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -710,7 +931,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A117"/>
+  <dimension ref="A1:A187"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
@@ -1298,7 +1519,361 @@
         <v>116</v>
       </c>
     </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A118" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A119" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A120" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A121" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A122" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A123" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A124" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A125" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A126" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A127" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A128" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A129" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A130" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A131" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A132" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A133" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A134" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="135" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A135" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="136" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A136" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="137" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A137" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="138" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A138" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="139" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A139" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="140" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A140" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="141" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A141" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="142" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A142" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="143" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A143" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="144" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A144" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A145" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="146" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A146" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="147" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A147" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="148" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A148" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="149" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A149" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="150" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A150" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="151" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A151" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="152" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A152" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="153" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A153" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="154" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A154" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="155" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A155" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="156" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A156" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="157" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A157" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="158" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A158" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="159" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A159" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="160" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A160" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="161" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A161" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="162" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A162" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="163" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A163" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="164" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A164" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="165" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A165" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="166" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A166" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="167" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A167" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="168" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A168" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="169" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A169" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="170" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A170" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="171" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A171" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="172" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A172" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="173" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A173" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="174" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A174" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="175" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A175" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="176" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A176" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="177" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A177" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="178" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A178" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="179" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A179" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="180" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A180" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="181" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A181" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="182" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A182" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="183" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A183" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="184" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A184" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="185" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A185" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="186" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A186" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="187" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A187" t="s">
+        <v>186</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A121" r:id="rId1" xr:uid="{DBCB34F7-13D5-4887-88B5-E5F9AE2C5B29}"/>
+    <hyperlink ref="A126" r:id="rId2" xr:uid="{1DFC794B-7257-4F35-B5FD-4D3E043ECEDC}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>